<commit_message>
actualizo generador de actas
</commit_message>
<xml_diff>
--- a/Generador de actas/acta_de_examen.xlsx
+++ b/Generador de actas/acta_de_examen.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection workbookPassword="C6D3" lockStructure="1"/>
+  <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -57,13 +57,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -430,57 +427,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ALUMNO</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>DNI</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MODALIDAD</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>CONDICION</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>CURSO</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ESPACIO CURRICULAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AMIRA YARBOUH</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>17599256</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MMO</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1°1°</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>GEOGRAFÍA I</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="C6D3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -491,52 +511,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ALUMNO</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>DNI</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MODALIDAD</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>CONDICION</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>CURSO</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ESPACIO CURRICULAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AMIRA YARBOUH</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>17599256</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MMO</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1°1°</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>GEOGRAFÍA I</t>
         </is>
       </c>
     </row>
@@ -551,52 +595,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ALUMNO</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>DNI</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>MODALIDAD</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>CONDICION</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>CURSO</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ESPACIO CURRICULAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AMIRA YARBOUH</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>17599256</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MMO</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1°1°</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>GEOGRAFÍA I</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
agrego para agregar materias
</commit_message>
<xml_diff>
--- a/Generador de actas/acta_de_examen.xlsx
+++ b/Generador de actas/acta_de_examen.xlsx
@@ -57,10 +57,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,78 +435,92 @@
   </sheetPr>
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>ALUMNO</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>DNI</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>MODALIDAD</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>CONDICION</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>CURSO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>ESPACIO CURRICULAR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>AMIRA YARBOUH</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>17599256</v>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>17599256</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>MMO</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>1°1°</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>GEOGRAFÍA I</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="C6D3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -513,72 +533,85 @@
   </sheetPr>
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>ALUMNO</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>DNI</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>MODALIDAD</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>CONDICION</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>CURSO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>ESPACIO CURRICULAR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>AMIRA YARBOUH</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>17599256</v>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>17599256</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>MMO</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>1°1°</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>GEOGRAFÍA I</t>
         </is>
@@ -597,72 +630,85 @@
   </sheetPr>
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>ALUMNO</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>DNI</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>MODALIDAD</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>CONDICION</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>CURSO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>ESPACIO CURRICULAR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>AMIRA YARBOUH</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>17599256</v>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>17599256</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>MMO</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>REGULAR</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>1°1°</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>GEOGRAFÍA I</t>
         </is>

</xml_diff>